<commit_message>
deleted the copy slide
</commit_message>
<xml_diff>
--- a/SFN/covariates/activationXageC16.xlsx
+++ b/SFN/covariates/activationXageC16.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avidachs/Documents/GitHub/rf1-sra-trust/SFN/Images/Graphs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avidachs/Documents/GitHub/rf1-sra-trust/SFN/covariates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60641EBA-EC77-9943-80CC-D7E8E0BA8CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66C22F2-7E80-1841-ACD1-B17D36237688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{237D927A-4980-744D-8F94-C4A707B37354}"/>
+    <workbookView xWindow="4140" yWindow="1880" windowWidth="28800" windowHeight="16120" xr2:uid="{237D927A-4980-744D-8F94-C4A707B37354}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,10 +41,10 @@
     <t>age</t>
   </si>
   <si>
-    <t>acc</t>
+    <t>mPFC</t>
   </si>
   <si>
-    <t>c17</t>
+    <t>dlPFC</t>
   </si>
 </sst>
 </file>
@@ -413,7 +413,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="9.1640625" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
@@ -422,10 +422,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -433,10 +433,10 @@
         <v>35.94</v>
       </c>
       <c r="B2" s="2">
+        <v>23.917718709999999</v>
+      </c>
+      <c r="C2" s="2">
         <v>42.117870920000001</v>
-      </c>
-      <c r="C2" s="2">
-        <v>23.917718709999999</v>
       </c>
       <c r="G2" s="1"/>
     </row>
@@ -445,10 +445,10 @@
         <v>68.64</v>
       </c>
       <c r="B3" s="2">
+        <v>103.87257820000001</v>
+      </c>
+      <c r="C3" s="2">
         <v>36.907285850000001</v>
-      </c>
-      <c r="C3" s="2">
-        <v>103.87257820000001</v>
       </c>
       <c r="G3" s="1"/>
     </row>
@@ -457,10 +457,10 @@
         <v>27.9</v>
       </c>
       <c r="B4" s="2">
+        <v>-33.601144869999999</v>
+      </c>
+      <c r="C4" s="2">
         <v>4.2015192030000001</v>
-      </c>
-      <c r="C4" s="2">
-        <v>-33.601144869999999</v>
       </c>
       <c r="G4" s="1"/>
     </row>
@@ -469,10 +469,10 @@
         <v>67.8</v>
       </c>
       <c r="B5" s="2">
+        <v>207.8942907</v>
+      </c>
+      <c r="C5" s="2">
         <v>-49.926510620000002</v>
-      </c>
-      <c r="C5" s="2">
-        <v>207.8942907</v>
       </c>
       <c r="G5" s="1"/>
     </row>
@@ -481,10 +481,10 @@
         <v>69.16</v>
       </c>
       <c r="B6" s="2">
+        <v>-23.037789549999999</v>
+      </c>
+      <c r="C6" s="2">
         <v>-41.233315040000001</v>
-      </c>
-      <c r="C6" s="2">
-        <v>-23.037789549999999</v>
       </c>
       <c r="G6" s="1"/>
     </row>
@@ -493,10 +493,10 @@
         <v>70.459999999999994</v>
       </c>
       <c r="B7" s="2">
+        <v>4.4514377620000003</v>
+      </c>
+      <c r="C7" s="2">
         <v>-112.16538679999999</v>
-      </c>
-      <c r="C7" s="2">
-        <v>4.4514377620000003</v>
       </c>
       <c r="G7" s="1"/>
     </row>
@@ -505,10 +505,10 @@
         <v>48.03</v>
       </c>
       <c r="B8" s="2">
+        <v>252.6476304</v>
+      </c>
+      <c r="C8" s="2">
         <v>134.61040320000001</v>
-      </c>
-      <c r="C8" s="2">
-        <v>252.6476304</v>
       </c>
       <c r="G8" s="1"/>
     </row>
@@ -517,10 +517,10 @@
         <v>49.64</v>
       </c>
       <c r="B9" s="2">
+        <v>71.643603880000001</v>
+      </c>
+      <c r="C9" s="2">
         <v>-9.183310251</v>
-      </c>
-      <c r="C9" s="2">
-        <v>71.643603880000001</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -529,10 +529,10 @@
         <v>63.33</v>
       </c>
       <c r="B10" s="2">
+        <v>267.68042050000003</v>
+      </c>
+      <c r="C10" s="2">
         <v>22.711778429999999</v>
-      </c>
-      <c r="C10" s="2">
-        <v>267.68042050000003</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -541,10 +541,10 @@
         <v>34.869999999999997</v>
       </c>
       <c r="B11" s="2">
+        <v>91.865850050000006</v>
+      </c>
+      <c r="C11" s="2">
         <v>138.87169019999999</v>
-      </c>
-      <c r="C11" s="2">
-        <v>91.865850050000006</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -553,10 +553,10 @@
         <v>56.4</v>
       </c>
       <c r="B12" s="2">
+        <v>76.707787969999998</v>
+      </c>
+      <c r="C12" s="2">
         <v>95.349950509999999</v>
-      </c>
-      <c r="C12" s="2">
-        <v>76.707787969999998</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -565,10 +565,10 @@
         <v>27.27</v>
       </c>
       <c r="B13" s="2">
+        <v>30.652052229999999</v>
+      </c>
+      <c r="C13" s="2">
         <v>123.1628982</v>
-      </c>
-      <c r="C13" s="2">
-        <v>30.652052229999999</v>
       </c>
       <c r="G13" s="1"/>
     </row>
@@ -577,10 +577,10 @@
         <v>69.22</v>
       </c>
       <c r="B14" s="2">
+        <v>-16.960082150000002</v>
+      </c>
+      <c r="C14" s="2">
         <v>15.57103554</v>
-      </c>
-      <c r="C14" s="2">
-        <v>-16.960082150000002</v>
       </c>
       <c r="G14" s="1"/>
     </row>
@@ -589,10 +589,10 @@
         <v>22.4</v>
       </c>
       <c r="B15" s="2">
+        <v>14.547055370000001</v>
+      </c>
+      <c r="C15" s="2">
         <v>207.2262332</v>
-      </c>
-      <c r="C15" s="2">
-        <v>14.547055370000001</v>
       </c>
       <c r="G15" s="1"/>
     </row>
@@ -601,10 +601,10 @@
         <v>26.81</v>
       </c>
       <c r="B16" s="2">
+        <v>93.526465630000004</v>
+      </c>
+      <c r="C16" s="2">
         <v>42.805273900000003</v>
-      </c>
-      <c r="C16" s="2">
-        <v>93.526465630000004</v>
       </c>
       <c r="G16" s="1"/>
     </row>
@@ -613,10 +613,10 @@
         <v>71.83</v>
       </c>
       <c r="B17" s="2">
+        <v>-24.984880799999999</v>
+      </c>
+      <c r="C17" s="2">
         <v>-25.033402850000002</v>
-      </c>
-      <c r="C17" s="2">
-        <v>-24.984880799999999</v>
       </c>
       <c r="G17" s="1"/>
     </row>
@@ -625,10 +625,10 @@
         <v>31.73</v>
       </c>
       <c r="B18" s="2">
+        <v>-67.126932749999995</v>
+      </c>
+      <c r="C18" s="2">
         <v>-73.249672360000005</v>
-      </c>
-      <c r="C18" s="2">
-        <v>-67.126932749999995</v>
       </c>
       <c r="G18" s="1"/>
     </row>
@@ -637,10 +637,10 @@
         <v>31.9</v>
       </c>
       <c r="B19" s="2">
+        <v>31.42278971</v>
+      </c>
+      <c r="C19" s="2">
         <v>-42.23875915</v>
-      </c>
-      <c r="C19" s="2">
-        <v>31.42278971</v>
       </c>
       <c r="G19" s="1"/>
     </row>
@@ -649,10 +649,10 @@
         <v>69.41</v>
       </c>
       <c r="B20" s="2">
+        <v>82.004579669999998</v>
+      </c>
+      <c r="C20" s="2">
         <v>-9.970225868</v>
-      </c>
-      <c r="C20" s="2">
-        <v>82.004579669999998</v>
       </c>
       <c r="G20" s="1"/>
     </row>
@@ -661,10 +661,10 @@
         <v>24.59</v>
       </c>
       <c r="B21" s="2">
+        <v>-78.7618358</v>
+      </c>
+      <c r="C21" s="2">
         <v>100.9959795</v>
-      </c>
-      <c r="C21" s="2">
-        <v>-78.7618358</v>
       </c>
       <c r="G21" s="1"/>
     </row>
@@ -673,10 +673,10 @@
         <v>63.8</v>
       </c>
       <c r="B22" s="2">
+        <v>141.4894577</v>
+      </c>
+      <c r="C22" s="2">
         <v>157.59621949999999</v>
-      </c>
-      <c r="C22" s="2">
-        <v>141.4894577</v>
       </c>
       <c r="G22" s="1"/>
     </row>
@@ -685,10 +685,10 @@
         <v>70.05</v>
       </c>
       <c r="B23" s="2">
+        <v>156.88871040000001</v>
+      </c>
+      <c r="C23" s="2">
         <v>-64.337306749999996</v>
-      </c>
-      <c r="C23" s="2">
-        <v>156.88871040000001</v>
       </c>
       <c r="G23" s="1"/>
     </row>
@@ -697,10 +697,10 @@
         <v>21.43</v>
       </c>
       <c r="B24" s="2">
+        <v>-265.44976159999999</v>
+      </c>
+      <c r="C24" s="2">
         <v>148.1257938</v>
-      </c>
-      <c r="C24" s="2">
-        <v>-265.44976159999999</v>
       </c>
       <c r="G24" s="1"/>
     </row>
@@ -709,10 +709,10 @@
         <v>62.39</v>
       </c>
       <c r="B25" s="2">
+        <v>106.8057091</v>
+      </c>
+      <c r="C25" s="2">
         <v>-267.14190880000001</v>
-      </c>
-      <c r="C25" s="2">
-        <v>106.8057091</v>
       </c>
       <c r="G25" s="1"/>
     </row>
@@ -721,10 +721,10 @@
         <v>22.07</v>
       </c>
       <c r="B26" s="2">
+        <v>-46.655395460000001</v>
+      </c>
+      <c r="C26" s="2">
         <v>387.39459849999997</v>
-      </c>
-      <c r="C26" s="2">
-        <v>-46.655395460000001</v>
       </c>
       <c r="G26" s="1"/>
     </row>
@@ -733,10 +733,10 @@
         <v>48.6</v>
       </c>
       <c r="B27" s="2">
+        <v>3.377600921</v>
+      </c>
+      <c r="C27" s="2">
         <v>280.7953321</v>
-      </c>
-      <c r="C27" s="2">
-        <v>3.377600921</v>
       </c>
       <c r="G27" s="1"/>
     </row>
@@ -745,10 +745,10 @@
         <v>33.200000000000003</v>
       </c>
       <c r="B28" s="2">
+        <v>-174.26956060000001</v>
+      </c>
+      <c r="C28" s="2">
         <v>70.882656060000002</v>
-      </c>
-      <c r="C28" s="2">
-        <v>-174.26956060000001</v>
       </c>
       <c r="G28" s="1"/>
     </row>
@@ -757,10 +757,10 @@
         <v>33.369999999999997</v>
       </c>
       <c r="B29" s="2">
+        <v>-22.574252609999998</v>
+      </c>
+      <c r="C29" s="2">
         <v>55.897045249999998</v>
-      </c>
-      <c r="C29" s="2">
-        <v>-22.574252609999998</v>
       </c>
       <c r="G29" s="1"/>
     </row>
@@ -769,10 +769,10 @@
         <v>34.43</v>
       </c>
       <c r="B30" s="2">
+        <v>-14.6959985</v>
+      </c>
+      <c r="C30" s="2">
         <v>76.170424519999997</v>
-      </c>
-      <c r="C30" s="2">
-        <v>-14.6959985</v>
       </c>
       <c r="G30" s="1"/>
     </row>
@@ -781,10 +781,10 @@
         <v>58.27</v>
       </c>
       <c r="B31" s="2">
+        <v>161.8278713</v>
+      </c>
+      <c r="C31" s="2">
         <v>-161.56934480000001</v>
-      </c>
-      <c r="C31" s="2">
-        <v>161.8278713</v>
       </c>
       <c r="G31" s="1"/>
     </row>
@@ -793,10 +793,10 @@
         <v>23.61</v>
       </c>
       <c r="B32" s="2">
+        <v>73.306786939999995</v>
+      </c>
+      <c r="C32" s="2">
         <v>81.144687160000004</v>
-      </c>
-      <c r="C32" s="2">
-        <v>73.306786939999995</v>
       </c>
       <c r="G32" s="1"/>
     </row>
@@ -805,10 +805,10 @@
         <v>27.02</v>
       </c>
       <c r="B33" s="2">
+        <v>-97.028571330000005</v>
+      </c>
+      <c r="C33" s="2">
         <v>331.05135899999999</v>
-      </c>
-      <c r="C33" s="2">
-        <v>-97.028571330000005</v>
       </c>
       <c r="G33" s="1"/>
     </row>
@@ -817,10 +817,10 @@
         <v>69.13</v>
       </c>
       <c r="B34" s="2">
+        <v>169.34094959999999</v>
+      </c>
+      <c r="C34" s="2">
         <v>20.109649009999998</v>
-      </c>
-      <c r="C34" s="2">
-        <v>169.34094959999999</v>
       </c>
       <c r="G34" s="1"/>
     </row>
@@ -829,10 +829,10 @@
         <v>28.3</v>
       </c>
       <c r="B35" s="2">
+        <v>-128.2470041</v>
+      </c>
+      <c r="C35" s="2">
         <v>268.07176420000002</v>
-      </c>
-      <c r="C35" s="2">
-        <v>-128.2470041</v>
       </c>
       <c r="G35" s="1"/>
     </row>
@@ -841,10 +841,10 @@
         <v>33.44</v>
       </c>
       <c r="B36" s="2">
+        <v>-27.0306803</v>
+      </c>
+      <c r="C36" s="2">
         <v>114.454903</v>
-      </c>
-      <c r="C36" s="2">
-        <v>-27.0306803</v>
       </c>
       <c r="G36" s="1"/>
     </row>
@@ -853,10 +853,10 @@
         <v>21.7</v>
       </c>
       <c r="B37" s="2">
+        <v>-54.524705789999999</v>
+      </c>
+      <c r="C37" s="2">
         <v>119.3642159</v>
-      </c>
-      <c r="C37" s="2">
-        <v>-54.524705789999999</v>
       </c>
       <c r="G37" s="1"/>
     </row>
@@ -865,10 +865,10 @@
         <v>36.93</v>
       </c>
       <c r="B38" s="2">
+        <v>151.2231773</v>
+      </c>
+      <c r="C38" s="2">
         <v>122.7957167</v>
-      </c>
-      <c r="C38" s="2">
-        <v>151.2231773</v>
       </c>
       <c r="G38" s="1"/>
     </row>
@@ -877,10 +877,10 @@
         <v>33.299999999999997</v>
       </c>
       <c r="B39" s="2">
+        <v>-43.418290919999997</v>
+      </c>
+      <c r="C39" s="2">
         <v>151.28646620000001</v>
-      </c>
-      <c r="C39" s="2">
-        <v>-43.418290919999997</v>
       </c>
       <c r="G39" s="1"/>
     </row>
@@ -889,10 +889,10 @@
         <v>25.51</v>
       </c>
       <c r="B40" s="2">
+        <v>-302.4211474</v>
+      </c>
+      <c r="C40" s="2">
         <v>305.6515488</v>
-      </c>
-      <c r="C40" s="2">
-        <v>-302.4211474</v>
       </c>
       <c r="G40" s="1"/>
     </row>
@@ -901,10 +901,10 @@
         <v>64.52</v>
       </c>
       <c r="B41" s="2">
+        <v>-20.209015749999999</v>
+      </c>
+      <c r="C41" s="2">
         <v>-131.97685139999999</v>
-      </c>
-      <c r="C41" s="2">
-        <v>-20.209015749999999</v>
       </c>
       <c r="G41" s="1"/>
     </row>
@@ -913,10 +913,10 @@
         <v>37.53</v>
       </c>
       <c r="B42" s="2">
+        <v>165.0671715</v>
+      </c>
+      <c r="C42" s="2">
         <v>236.62153029999999</v>
-      </c>
-      <c r="C42" s="2">
-        <v>165.0671715</v>
       </c>
       <c r="G42" s="1"/>
     </row>
@@ -925,10 +925,10 @@
         <v>51.18</v>
       </c>
       <c r="B43" s="2">
+        <v>21.02857818</v>
+      </c>
+      <c r="C43" s="2">
         <v>183.96061449999999</v>
-      </c>
-      <c r="C43" s="2">
-        <v>21.02857818</v>
       </c>
       <c r="G43" s="1"/>
     </row>
@@ -937,10 +937,10 @@
         <v>61.23</v>
       </c>
       <c r="B44" s="2">
+        <v>8.1231475500000005</v>
+      </c>
+      <c r="C44" s="2">
         <v>-76.842516099999997</v>
-      </c>
-      <c r="C44" s="2">
-        <v>8.1231475500000005</v>
       </c>
       <c r="G44" s="1"/>
     </row>
@@ -949,10 +949,10 @@
         <v>39.69</v>
       </c>
       <c r="B45" s="2">
+        <v>57.241111240000002</v>
+      </c>
+      <c r="C45" s="2">
         <v>233.14218360000001</v>
-      </c>
-      <c r="C45" s="2">
-        <v>57.241111240000002</v>
       </c>
       <c r="G45" s="1"/>
     </row>
@@ -961,10 +961,10 @@
         <v>26.85</v>
       </c>
       <c r="B46" s="2">
+        <v>29.740692330000002</v>
+      </c>
+      <c r="C46" s="2">
         <v>204.745214</v>
-      </c>
-      <c r="C46" s="2">
-        <v>29.740692330000002</v>
       </c>
       <c r="G46" s="1"/>
     </row>
@@ -973,10 +973,10 @@
         <v>34.53</v>
       </c>
       <c r="B47" s="2">
+        <v>-40.998753049999998</v>
+      </c>
+      <c r="C47" s="2">
         <v>114.92957970000001</v>
-      </c>
-      <c r="C47" s="2">
-        <v>-40.998753049999998</v>
       </c>
       <c r="G47" s="1"/>
     </row>
@@ -985,10 +985,10 @@
         <v>42.69</v>
       </c>
       <c r="B48" s="2">
+        <v>70.614622249999996</v>
+      </c>
+      <c r="C48" s="2">
         <v>128.61670570000001</v>
-      </c>
-      <c r="C48" s="2">
-        <v>70.614622249999996</v>
       </c>
       <c r="G48" s="1"/>
     </row>
@@ -997,10 +997,10 @@
         <v>25.5</v>
       </c>
       <c r="B49" s="2">
+        <v>-155.6357232</v>
+      </c>
+      <c r="C49" s="2">
         <v>224.30717469999999</v>
-      </c>
-      <c r="C49" s="2">
-        <v>-155.6357232</v>
       </c>
       <c r="G49" s="1"/>
     </row>
@@ -1009,10 +1009,10 @@
         <v>26.99</v>
       </c>
       <c r="B50" s="2">
+        <v>-73.615104419999994</v>
+      </c>
+      <c r="C50" s="2">
         <v>561.50802759999999</v>
-      </c>
-      <c r="C50" s="2">
-        <v>-73.615104419999994</v>
       </c>
       <c r="G50" s="1"/>
     </row>
@@ -1021,10 +1021,10 @@
         <v>58.05</v>
       </c>
       <c r="B51" s="2">
+        <v>53.404600719999998</v>
+      </c>
+      <c r="C51" s="2">
         <v>27.897000269999999</v>
-      </c>
-      <c r="C51" s="2">
-        <v>53.404600719999998</v>
       </c>
       <c r="G51" s="1"/>
     </row>
@@ -1033,10 +1033,10 @@
         <v>68.77</v>
       </c>
       <c r="B52" s="2">
+        <v>99.914298160000001</v>
+      </c>
+      <c r="C52" s="2">
         <v>26.09479984</v>
-      </c>
-      <c r="C52" s="2">
-        <v>99.914298160000001</v>
       </c>
       <c r="G52" s="1"/>
     </row>
@@ -1045,10 +1045,10 @@
         <v>62.91</v>
       </c>
       <c r="B53" s="2">
+        <v>255.15375220000001</v>
+      </c>
+      <c r="C53" s="2">
         <v>268.05524800000001</v>
-      </c>
-      <c r="C53" s="2">
-        <v>255.15375220000001</v>
       </c>
       <c r="G53" s="1"/>
     </row>
@@ -1057,10 +1057,10 @@
         <v>62.96</v>
       </c>
       <c r="B54" s="2">
+        <v>-61.14925452</v>
+      </c>
+      <c r="C54" s="2">
         <v>-146.16520130000001</v>
-      </c>
-      <c r="C54" s="2">
-        <v>-61.14925452</v>
       </c>
       <c r="G54" s="1"/>
     </row>
@@ -1069,10 +1069,10 @@
         <v>31.95</v>
       </c>
       <c r="B55" s="2">
+        <v>-130.65157959999999</v>
+      </c>
+      <c r="C55" s="2">
         <v>102.3980756</v>
-      </c>
-      <c r="C55" s="2">
-        <v>-130.65157959999999</v>
       </c>
       <c r="G55" s="1"/>
     </row>
@@ -1081,10 +1081,10 @@
         <v>62.04</v>
       </c>
       <c r="B56" s="2">
+        <v>68.662003350000006</v>
+      </c>
+      <c r="C56" s="2">
         <v>-75.831739580000004</v>
-      </c>
-      <c r="C56" s="2">
-        <v>68.662003350000006</v>
       </c>
       <c r="G56" s="1"/>
     </row>
@@ -1093,10 +1093,10 @@
         <v>41.91</v>
       </c>
       <c r="B57" s="2">
+        <v>-68.761223340000001</v>
+      </c>
+      <c r="C57" s="2">
         <v>-291.69823609999997</v>
-      </c>
-      <c r="C57" s="2">
-        <v>-68.761223340000001</v>
       </c>
       <c r="G57" s="1"/>
     </row>
@@ -1105,10 +1105,10 @@
         <v>29.07</v>
       </c>
       <c r="B58" s="2">
+        <v>-15.30247144</v>
+      </c>
+      <c r="C58" s="2">
         <v>163.65182050000001</v>
-      </c>
-      <c r="C58" s="2">
-        <v>-15.30247144</v>
       </c>
       <c r="G58" s="1"/>
     </row>
@@ -1117,10 +1117,10 @@
         <v>73.400000000000006</v>
       </c>
       <c r="B59" s="2">
+        <v>-23.456584880000001</v>
+      </c>
+      <c r="C59" s="2">
         <v>74.161334420000003</v>
-      </c>
-      <c r="C59" s="2">
-        <v>-23.456584880000001</v>
       </c>
       <c r="G59" s="1"/>
     </row>
@@ -1129,10 +1129,10 @@
         <v>44.68</v>
       </c>
       <c r="B60" s="2">
+        <v>-116.9775471</v>
+      </c>
+      <c r="C60" s="2">
         <v>166.39815859999999</v>
-      </c>
-      <c r="C60" s="2">
-        <v>-116.9775471</v>
       </c>
       <c r="G60" s="1"/>
     </row>
@@ -1141,10 +1141,10 @@
         <v>58.98</v>
       </c>
       <c r="B61" s="2">
+        <v>17.93763246</v>
+      </c>
+      <c r="C61" s="2">
         <v>-6.1938781929999998</v>
-      </c>
-      <c r="C61" s="2">
-        <v>17.93763246</v>
       </c>
       <c r="G61" s="1"/>
     </row>
@@ -1153,10 +1153,10 @@
         <v>21.66</v>
       </c>
       <c r="B62" s="2">
+        <v>-72.566137510000004</v>
+      </c>
+      <c r="C62" s="2">
         <v>229.4641513</v>
-      </c>
-      <c r="C62" s="2">
-        <v>-72.566137510000004</v>
       </c>
       <c r="G62" s="1"/>
     </row>
@@ -1165,10 +1165,10 @@
         <v>38.36</v>
       </c>
       <c r="B63" s="2">
+        <v>-121.9706156</v>
+      </c>
+      <c r="C63" s="2">
         <v>101.34703620000001</v>
-      </c>
-      <c r="C63" s="2">
-        <v>-121.9706156</v>
       </c>
       <c r="G63" s="1"/>
     </row>

</xml_diff>